<commit_message>
fix: config CSRF + secret key via env
</commit_message>
<xml_diff>
--- a/Data/Exercices.xlsx
+++ b/Data/Exercices.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\sport-app\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\sport-app\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04CA7D3C-A279-4C18-9496-B68C9D3AB90F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D1FA93-53A4-4155-84E9-0CA04337B438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="550" yWindow="2170" windowWidth="15370" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="22660" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exercice" sheetId="13" r:id="rId1"/>
@@ -35,9 +35,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="40">
   <si>
-    <t>Presse inclinée pieds hauts</t>
-  </si>
-  <si>
     <t>Leg Curl</t>
   </si>
   <si>
@@ -153,6 +150,9 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t>Presse inclinée</t>
   </si>
 </sst>
 </file>
@@ -539,199 +539,199 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>

</xml_diff>